<commit_message>
Drop Dhanlaxmi Bank (low fit); add how-Zocket-helps notes for 19 new accounts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ABqraVRjb7dW9RHz2X61A
</commit_message>
<xml_diff>
--- a/tam/Zocket_TAM_Additions_v2.xlsx
+++ b/tam/Zocket_TAM_Additions_v2.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Add to TAM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 new – how Zocket helps" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,9 +56,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1536,32 +1540,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dhanlaxmi Bank Ltd</t>
+          <t>Galderma India Pvt Ltd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dhanlaxmi Bank</t>
+          <t>Galderma India</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Banking</t>
+          <t>Beauty, Personal Care &amp; Wellness</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.dhan.bank.in</t>
+          <t>https://www.galderma.com/india</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Thrissur</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1571,25 +1575,25 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>16,010,000,000</t>
+          <t>12,500,000,000</t>
         </is>
       </c>
       <c r="K17" t="n">
-        <v>1601</v>
+        <v>1250</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/DHANBANK/</t>
+          <t>https://www.tofler.in/galderma-india-private-limited/company/U24110MH1999PTC118113</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1604,12 +1608,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Galderma India Pvt Ltd</t>
+          <t>Pureplay Skin Sciences (India) Pvt Ltd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Galderma India</t>
+          <t>Plum</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1619,7 +1623,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.galderma.com/india</t>
+          <t>https://plumgoodness.com</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/plumgoodness</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1639,25 +1648,25 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>12,500,000,000</t>
+          <t>5,150,000,000</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>1250</v>
+        <v>515</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://www.tofler.in/galderma-india-private-limited/company/U24110MH1999PTC118113</t>
+          <t>https://entrackr.com/fintrackr/d2c-brand-plums-revenue-crosses-rs-500-cr-in-fy26-profit-doubles-12486368</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1672,37 +1681,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pureplay Skin Sciences (India) Pvt Ltd</t>
+          <t>Marwadi Shares and Finance Ltd</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Plum</t>
+          <t>Marwadi Financial Services</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Beauty, Personal Care &amp; Wellness</t>
+          <t>Broking &amp; Wealth</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://plumgoodness.com</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/plumgoodness</t>
+          <t>https://www.marwadionline.com</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Rajkot</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Maharashtra</t>
+          <t>Gujarat</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1712,20 +1716,20 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>5,150,000,000</t>
+          <t>8,911,000,000</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>515</v>
+        <v>891.1</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://entrackr.com/fintrackr/d2c-brand-plums-revenue-crosses-rs-500-cr-in-fy26-profit-doubles-12486368</t>
+          <t>https://infomericstorage.blob.core.windows.net/uploads/pr_Marwadi_Shares_20mar26_91ce494dfa.pdf</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1745,32 +1749,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Marwadi Shares and Finance Ltd</t>
+          <t>B New Mobiles Pvt Ltd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Marwadi Financial Services</t>
+          <t>B New Mobiles</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Broking &amp; Wealth</t>
+          <t>Consumer Electronics</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.marwadionline.com</t>
+          <t>https://bnewmobiles.com</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Rajkot</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Gujarat</t>
+          <t>Andhra Pradesh</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1780,11 +1784,11 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>8,911,000,000</t>
+          <t>12,500,000,000</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>891.1</v>
+        <v>1250</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1793,12 +1797,12 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://infomericstorage.blob.core.windows.net/uploads/pr_Marwadi_Shares_20mar26_91ce494dfa.pdf</t>
+          <t>https://www.tofler.in/b-new-mobiles-private-limited/company/U51226AP2014PTC095072</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1813,12 +1817,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>B New Mobiles Pvt Ltd</t>
+          <t>Prakash Retail Pvt Ltd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>B New Mobiles</t>
+          <t>Harsha</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1828,17 +1832,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://bnewmobiles.com</t>
+          <t>https://www.harshaonline.com</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Udupi</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1848,11 +1852,11 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>12,500,000,000</t>
+          <t>6,081,000,000</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>1250</v>
+        <v>608.1</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1861,17 +1865,17 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>https://www.tofler.in/b-new-mobiles-private-limited/company/U51226AP2014PTC095072</t>
+          <t>https://connect.acuite.in/fcompany-details/PRAKASH_RETAIL_PRIVATE_LIMITED/7th_Nov_25</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Tensai lookalike list</t>
+          <t>Earlier research</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1885,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Prakash Retail Pvt Ltd</t>
+          <t>Muthoottu Mini Financiers Ltd</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Harsha</t>
+          <t>Muthoottu Mini</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Consumer Electronics</t>
+          <t>Gold Loans &amp; Microfinance</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.harshaonline.com</t>
+          <t>https://www.muthoottumini.com</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Udupi</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Kerala</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1916,11 +1920,11 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>6,081,000,000</t>
+          <t>8,150,000,000</t>
         </is>
       </c>
       <c r="K22" t="n">
-        <v>608.1</v>
+        <v>815</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1929,7 +1933,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://connect.acuite.in/fcompany-details/PRAKASH_RETAIL_PRIVATE_LIMITED/7th_Nov_25</t>
+          <t>https://www.careratings.com/upload/CompanyFiles/PR/202507130710_Muthoottu_Mini_Financiers_Limited.pdf</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1939,7 +1943,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Earlier research</t>
+          <t>Tensai lookalike list</t>
         </is>
       </c>
     </row>
@@ -1949,12 +1953,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Muthoottu Mini Financiers Ltd</t>
+          <t>Indel Money Ltd</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Muthoottu Mini</t>
+          <t>Indel Money</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1964,7 +1968,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.muthoottumini.com</t>
+          <t>https://www.indelmoney.com</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1984,25 +1988,25 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>8,150,000,000</t>
+          <t>6,060,000,000</t>
         </is>
       </c>
       <c r="K23" t="n">
-        <v>815</v>
+        <v>606</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>https://www.careratings.com/upload/CompanyFiles/PR/202507130710_Muthoottu_Mini_Financiers_Limited.pdf</t>
+          <t>https://infomericstorage.blob.core.windows.net/uploads/PR_Indel_Money19_Dec25_a4f977a327.pdf</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2017,32 +2021,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Indel Money Ltd</t>
+          <t>Shubham Housing Development Finance Company Ltd</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Indel Money</t>
+          <t>Shubham Housing Finance</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Gold Loans &amp; Microfinance</t>
+          <t>Housing Finance</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.indelmoney.com</t>
+          <t>https://www.shubham.co</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Haryana</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2052,20 +2056,20 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>6,060,000,000</t>
+          <t>8,241,000,000</t>
         </is>
       </c>
       <c r="K24" t="n">
-        <v>606</v>
+        <v>824.1</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://infomericstorage.blob.core.windows.net/uploads/PR_Indel_Money19_Dec25_a4f977a327.pdf</t>
+          <t>https://inc42.com/company/shubham-housing-development-finance-company/financials/</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2085,32 +2089,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Shubham Housing Development Finance Company Ltd</t>
+          <t>Hari Prasad Gopi Krishna Saraf Pvt Ltd</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Shubham Housing Finance</t>
+          <t>Aisshpra Gems &amp; Jewels</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Housing Finance</t>
+          <t>Jewellery &amp; Watches</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.shubham.co</t>
+          <t>https://www.aisshpra.com</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>Lucknow</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Haryana</t>
+          <t>Uttar Pradesh</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2120,11 +2124,11 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>8,241,000,000</t>
+          <t>16,460,000,000</t>
         </is>
       </c>
       <c r="K25" t="n">
-        <v>824.1</v>
+        <v>1646</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -2133,12 +2137,12 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>https://inc42.com/company/shubham-housing-development-finance-company/financials/</t>
+          <t>https://www.careratings.com/upload/CompanyFiles/PR/202603140327_HARI_PRASAD_GOPI_KRISHNA_SARAF_PRIVATE_LIMITED.pdf</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2153,12 +2157,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Hari Prasad Gopi Krishna Saraf Pvt Ltd</t>
+          <t>Arundhati Jewellers Pvt Ltd</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Aisshpra Gems &amp; Jewels</t>
+          <t>Arundhati Jewellers</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2168,17 +2172,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.aisshpra.com</t>
+          <t>https://www.arundhatijewellers.com</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Lucknow</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Uttar Pradesh</t>
+          <t>Odisha</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2188,25 +2192,25 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>16,460,000,000</t>
+          <t>8,030,000,000</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>1646</v>
+        <v>803</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>https://www.careratings.com/upload/CompanyFiles/PR/202603140327_HARI_PRASAD_GOPI_KRISHNA_SARAF_PRIVATE_LIMITED.pdf</t>
+          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=141534</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2221,32 +2225,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Arundhati Jewellers Pvt Ltd</t>
+          <t>Five-Star Business Finance Ltd</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Arundhati Jewellers</t>
+          <t>Five-Star Business Finance</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Jewellery &amp; Watches</t>
+          <t>NBFC &amp; Consumer Lending</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.arundhatijewellers.com</t>
+          <t>https://www.fivestargroup.in</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Odisha</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2256,25 +2260,25 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>8,030,000,000</t>
+          <t>28,480,000,000</t>
         </is>
       </c>
       <c r="K27" t="n">
-        <v>803</v>
+        <v>2848</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=141534</t>
+          <t>https://filingreader.com/news-wire/mumbai/2025-04-30/five-star-business-finance-announces-strong-fy25-results-conference-call</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2289,12 +2293,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Five-Star Business Finance Ltd</t>
+          <t>Branch International Financial Services Pvt Ltd</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Five-Star Business Finance</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2304,17 +2308,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.fivestargroup.in</t>
+          <t>https://branch.co.in</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Tamil Nadu</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2324,11 +2328,11 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>28,480,000,000</t>
+          <t>8,320,000,000</t>
         </is>
       </c>
       <c r="K28" t="n">
-        <v>2848</v>
+        <v>832</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -2337,12 +2341,12 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>https://filingreader.com/news-wire/mumbai/2025-04-30/five-star-business-finance-announces-strong-fy25-results-conference-call</t>
+          <t>https://tracxn.com/d/legal-entities/india/branch-international-financial-services-private-limited/__d-H872WiN20gk3Rth1kQjhTc7pu2iy49u4e-85thrao</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2357,32 +2361,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Branch International Financial Services Pvt Ltd</t>
+          <t>Darling Retail Pvt Ltd</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Darling Retail</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NBFC &amp; Consumer Lending</t>
+          <t>Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://branch.co.in</t>
+          <t>https://darlingretail.com</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2392,20 +2396,20 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>8,320,000,000</t>
+          <t>9,740,000,000</t>
         </is>
       </c>
       <c r="K29" t="n">
-        <v>832</v>
+        <v>974</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>https://tracxn.com/d/legal-entities/india/branch-international-financial-services-private-limited/__d-H872WiN20gk3Rth1kQjhTc7pu2iy49u4e-85thrao</t>
+          <t>https://www.icra.in/Rating/ShowRationalReportFilePdf/121014</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2425,130 +2429,419 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Darling Retail Pvt Ltd</t>
+          <t>Star Automobiles</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>Star Automobiles (Mahindra / Hero)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Auto Dealerships</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Jabalpur</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>9,906,000,000</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>990.6</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>https://www.icra.in/Rating/ShowRationalReportFilePdf/138597</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Earlier research</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>How Zocket helps</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aisshpra Gems &amp; Jewels</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Jewellery retail</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain holds brand rules, hallmark/BIS claims and offer terms. Creative AI produces festive and wedding creatives per showroom and language. Consumer AI tracks reviews and replies on Google listings. Paid Media AI shows which showroom campaigns bring walk-ins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Arundhati Jewellers</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Jewellery retail</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain holds brand rules, hallmark/BIS claims and offer terms. Creative AI produces festive and wedding creatives per showroom and language. Consumer AI tracks reviews and replies on Google listings. Paid Media AI shows which showroom campaigns bring walk-ins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>JG Hosiery (Amul Macho, Sporto)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Innerwear/apparel brands</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Paid Media AI handles big multi-brand budgets across TV-led digital. Creative AI produces many variants per SKU and festival, on brand. Consumer AI tracks share of voice against Rupa, Lux and Jockey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OTTO Clothing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Menswear brand</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Creative AI scales ad and marketplace creative for every collection drop. Paid Media AI optimises D2C and marketplace ads. Consumer AI reads reviews for fit and quality issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Plum (Pureplay Skin Sciences)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>D2C beauty</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Paid Media AI cuts wasted spend from creative fatigue across Meta and Google. Creative AI handles high-volume UGC-style and per-SKU creatives with claims checked. Consumer AI covers marketplace reviews.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Galderma India (Cetaphil)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Consumer skincare</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain enforces dermatology claims and disclaimers. Creative AI produces compliant creative for each SKU. Consumer AI covers reviews and sentiment across Nykaa, Amazon and social.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B New Mobiles</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mobile and electronics retail</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Consumer AI moderates reviews and inbox for 150 stores. Creative AI makes offer creatives for each store, in Telugu and English. Paid Media AI joins store footfall to ad spend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Darling Retail</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Retail &amp; E-commerce</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>https://darlingretail.com</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Tamil Nadu</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>9,740,000,000</t>
-        </is>
-      </c>
-      <c r="K30" t="n">
-        <v>974</v>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>https://www.icra.in/Rating/ShowRationalReportFilePdf/121014</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Tensai lookalike list</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Star Automobiles</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Star Automobiles (Mahindra / Hero)</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Auto Dealerships</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Jabalpur</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Madhya Pradesh</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>9,906,000,000</t>
-        </is>
-      </c>
-      <c r="K31" t="n">
-        <v>990.6</v>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>https://www.icra.in/Rating/ShowRationalReportFilePdf/138597</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Earlier research</t>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Electronics/furniture retail</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Consumer AI handles reviews across 185 stores. Creative AI makes local Tamil offer and festive creatives at scale. Paid Media AI handles store-level campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Galaxy Toyota</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Car dealer</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain keeps OEM brand rules for every outlet. Creative AI makes localised offer creatives per showroom. Paid Media AI cuts lead-ad waste and shows cost per test-drive. Consumer AI watches Google reviews for every outlet and replies to them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kataria Automobiles</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Car dealer group</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain keeps OEM brand rules for every outlet. Creative AI makes localised offer creatives per showroom. Paid Media AI cuts lead-ad waste and shows cost per test-drive. Consumer AI watches Google reviews for every outlet and replies to them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kalyani Motors</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Car dealer group</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain keeps OEM brand rules for every outlet. Creative AI makes localised offer creatives per showroom. Paid Media AI cuts lead-ad waste and shows cost per test-drive. Consumer AI watches Google reviews for every outlet and replies to them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bhandari Automobiles</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Car dealer group</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain keeps OEM brand rules for every outlet. Creative AI makes localised offer creatives per showroom. Paid Media AI cuts lead-ad waste and shows cost per test-drive. Consumer AI watches Google reviews for every outlet and replies to them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AMP Motors (JLR)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Luxury car dealer</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain enforces JLR luxury brand rules. Creative AI makes premium, on-brand local creative. Paid Media AI targets high-income buyers and tracks cost per test-drive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Five-Star Business Finance</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Small-business loans</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain locks RBI disclaimers and rate rules. Creative AI makes branch-level, multi-language ads without compliance slips. Paid Media AI optimises lead cost. Consumer AI handles complaints and reviews. Covers 700+ branches in regional languages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Marwadi Shares &amp; Finance</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Retail broking app</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Creative AI produces content and SEO at volume within SEBI rules. Paid Media AI optimises cost per app install and per active trader. Consumer AI covers app-store reviews and complaints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Branch International</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Personal-loan app</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Paid Media AI optimises cost per install and per approved loan. Creative AI produces fast ad variants with RBI disclaimers checked. Consumer AI covers Play Store reviews and grievances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Shubham Housing Finance</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Affordable home loans</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain locks RBI disclaimers and rate rules. Creative AI makes branch-level, multi-language ads without compliance slips. Paid Media AI optimises lead cost. Consumer AI handles complaints and reviews. Built for tier-2 and tier-3 markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Muthoottu Mini Financiers</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Gold loans</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain locks RBI disclaimers and rate rules. Creative AI makes branch-level, multi-language ads without compliance slips. Paid Media AI optimises lead cost. Consumer AI handles complaints and reviews. Covers 948 branches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Indel Money</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gold loans</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Brand Brain locks RBI disclaimers and rate rules. Creative AI makes branch-level, multi-language ads without compliance slips. Paid Media AI optimises lead cost. Consumer AI handles complaints and reviews. Covers 397 branches in 12 states.</t>
         </is>
       </c>
     </row>

</xml_diff>